<commit_message>
finished Sprint 7 docs
</commit_message>
<xml_diff>
--- a/doc/April 8th/COSC471PerformanceSchedule_4_8.xlsx
+++ b/doc/April 8th/COSC471PerformanceSchedule_4_8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\471 Project Repo\the-project-data-warehouse-team\doc\April 8th\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37996B2-9E6C-45CD-BEB0-77388F308B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FEBC20E-02CE-4220-93C5-26678B92A3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -829,7 +829,7 @@
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="9">
-        <v>1.1000000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="15"/>
@@ -841,7 +841,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="17"/>
@@ -865,7 +865,7 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="6">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="17"/>

</xml_diff>